<commit_message>
♻️ refactor: [no-ref] Replace rebate threshold with per-product VAT checkbox
- replace global rebate threshold with per-product "Usar preço c/ IVA" checkbox
- add `usar_iva` column to catalog: checked uses gross cost, unchecked uses net cost
- initialize missing flags once from legacy threshold rule (gross > limit → checked)
- remove threshold input from rebates UI; checkbox now controls cost basis per product
- add checkbox column to catalog editor with tooltip explaining behavior
- update reb
</commit_message>
<xml_diff>
--- a/static/catalogo.xlsx
+++ b/static/catalogo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>Preço total</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Usar preço c/ IVA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -473,6 +478,9 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -492,6 +500,9 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -511,6 +522,9 @@
       <c r="E4" t="n">
         <v>0</v>
       </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -530,6 +544,9 @@
       <c r="E5" t="n">
         <v>0</v>
       </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -549,6 +566,9 @@
       <c r="E6" t="n">
         <v>0</v>
       </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -568,6 +588,9 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -587,6 +610,9 @@
       <c r="E8" t="n">
         <v>0</v>
       </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -606,6 +632,9 @@
       <c r="E9" t="n">
         <v>58.19</v>
       </c>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -625,6 +654,9 @@
       <c r="E10" t="n">
         <v>12.1</v>
       </c>
+      <c r="F10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -644,6 +676,9 @@
       <c r="E11" t="n">
         <v>60.5</v>
       </c>
+      <c r="F11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -663,6 +698,9 @@
       <c r="E12" t="n">
         <v>12.1</v>
       </c>
+      <c r="F12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -682,6 +720,9 @@
       <c r="E13" t="n">
         <v>60.5</v>
       </c>
+      <c r="F13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -701,6 +742,9 @@
       <c r="E14" t="n">
         <v>16.5</v>
       </c>
+      <c r="F14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -720,6 +764,9 @@
       <c r="E15" t="n">
         <v>27.5</v>
       </c>
+      <c r="F15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -739,6 +786,9 @@
       <c r="E16" t="n">
         <v>22</v>
       </c>
+      <c r="F16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -758,6 +808,9 @@
       <c r="E17" t="n">
         <v>55</v>
       </c>
+      <c r="F17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -777,6 +830,9 @@
       <c r="E18" t="n">
         <v>11</v>
       </c>
+      <c r="F18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -796,6 +852,9 @@
       <c r="E19" t="n">
         <v>55</v>
       </c>
+      <c r="F19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -815,6 +874,9 @@
       <c r="E20" t="n">
         <v>220</v>
       </c>
+      <c r="F20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -834,6 +896,9 @@
       <c r="E21" t="n">
         <v>550</v>
       </c>
+      <c r="F21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -853,6 +918,9 @@
       <c r="E22" t="n">
         <v>8.199999999999999</v>
       </c>
+      <c r="F22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -872,6 +940,9 @@
       <c r="E23" t="n">
         <v>0</v>
       </c>
+      <c r="F23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -891,6 +962,9 @@
       <c r="E24" t="n">
         <v>0</v>
       </c>
+      <c r="F24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -910,6 +984,9 @@
       <c r="E25" t="n">
         <v>25.89</v>
       </c>
+      <c r="F25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -929,6 +1006,9 @@
       <c r="E26" t="n">
         <v>40.17</v>
       </c>
+      <c r="F26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -948,6 +1028,9 @@
       <c r="E27" t="n">
         <v>33.83</v>
       </c>
+      <c r="F27" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -967,6 +1050,9 @@
       <c r="E28" t="n">
         <v>56.21</v>
       </c>
+      <c r="F28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -986,6 +1072,9 @@
       <c r="E29" t="n">
         <v>30.81</v>
       </c>
+      <c r="F29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1005,6 +1094,9 @@
       <c r="E30" t="n">
         <v>46.74</v>
       </c>
+      <c r="F30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1024,6 +1116,9 @@
       <c r="E31" t="n">
         <v>40.28</v>
       </c>
+      <c r="F31" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1043,6 +1138,9 @@
       <c r="E32" t="n">
         <v>548.24</v>
       </c>
+      <c r="F32" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1062,6 +1160,9 @@
       <c r="E33" t="n">
         <v>301.8</v>
       </c>
+      <c r="F33" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1081,6 +1182,9 @@
       <c r="E34" t="n">
         <v>1173.75</v>
       </c>
+      <c r="F34" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1100,6 +1204,9 @@
       <c r="E35" t="n">
         <v>1443.71</v>
       </c>
+      <c r="F35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1119,6 +1226,9 @@
       <c r="E36" t="n">
         <v>4</v>
       </c>
+      <c r="F36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1138,6 +1248,9 @@
       <c r="E37" t="n">
         <v>358.84</v>
       </c>
+      <c r="F37" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1157,6 +1270,9 @@
       <c r="E38" t="n">
         <v>138.84</v>
       </c>
+      <c r="F38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1176,6 +1292,9 @@
       <c r="E39" t="n">
         <v>101.17</v>
       </c>
+      <c r="F39" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1195,6 +1314,9 @@
       <c r="E40" t="n">
         <v>53.14</v>
       </c>
+      <c r="F40" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1214,6 +1336,9 @@
       <c r="E41" t="n">
         <v>52.46</v>
       </c>
+      <c r="F41" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1233,6 +1358,9 @@
       <c r="E42" t="n">
         <v>147.85</v>
       </c>
+      <c r="F42" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1252,6 +1380,9 @@
       <c r="E43" t="n">
         <v>82.77</v>
       </c>
+      <c r="F43" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1271,6 +1402,9 @@
       <c r="E44" t="n">
         <v>55.35</v>
       </c>
+      <c r="F44" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1290,6 +1424,9 @@
       <c r="E45" t="n">
         <v>56.52</v>
       </c>
+      <c r="F45" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1309,6 +1446,9 @@
       <c r="E46" t="n">
         <v>463.76</v>
       </c>
+      <c r="F46" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1328,6 +1468,9 @@
       <c r="E47" t="n">
         <v>523.76</v>
       </c>
+      <c r="F47" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1347,6 +1490,9 @@
       <c r="E48" t="n">
         <v>110.07</v>
       </c>
+      <c r="F48" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1366,6 +1512,9 @@
       <c r="E49" t="n">
         <v>61.06</v>
       </c>
+      <c r="F49" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1385,6 +1534,9 @@
       <c r="E50" t="n">
         <v>239.07</v>
       </c>
+      <c r="F50" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1404,6 +1556,9 @@
       <c r="E51" t="n">
         <v>1000.07</v>
       </c>
+      <c r="F51" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1423,6 +1578,9 @@
       <c r="E52" t="n">
         <v>380.06</v>
       </c>
+      <c r="F52" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1442,6 +1600,9 @@
       <c r="E53" t="n">
         <v>47.06</v>
       </c>
+      <c r="F53" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1461,6 +1622,9 @@
       <c r="E54" t="n">
         <v>608.84</v>
       </c>
+      <c r="F54" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1480,6 +1644,9 @@
       <c r="E55" t="n">
         <v>86.06</v>
       </c>
+      <c r="F55" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1499,6 +1666,9 @@
       <c r="E56" t="n">
         <v>33.21</v>
       </c>
+      <c r="F56" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1518,6 +1688,9 @@
       <c r="E57" t="n">
         <v>57.06</v>
       </c>
+      <c r="F57" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1537,6 +1710,9 @@
       <c r="E58" t="n">
         <v>171.06</v>
       </c>
+      <c r="F58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1556,6 +1732,9 @@
       <c r="E59" t="n">
         <v>144.75</v>
       </c>
+      <c r="F59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1575,6 +1754,9 @@
       <c r="E60" t="n">
         <v>91.06</v>
       </c>
+      <c r="F60" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1594,6 +1776,9 @@
       <c r="E61" t="n">
         <v>91.06</v>
       </c>
+      <c r="F61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1613,6 +1798,9 @@
       <c r="E62" t="n">
         <v>37.1</v>
       </c>
+      <c r="F62" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1632,6 +1820,9 @@
       <c r="E63" t="n">
         <v>104.72</v>
       </c>
+      <c r="F63" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1651,6 +1842,9 @@
       <c r="E64" t="n">
         <v>99.72</v>
       </c>
+      <c r="F64" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1670,6 +1864,9 @@
       <c r="E65" t="n">
         <v>109.72</v>
       </c>
+      <c r="F65" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1689,6 +1886,9 @@
       <c r="E66" t="n">
         <v>100.97</v>
       </c>
+      <c r="F66" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1708,6 +1908,9 @@
       <c r="E67" t="n">
         <v>211.06</v>
       </c>
+      <c r="F67" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1727,6 +1930,9 @@
       <c r="E68" t="n">
         <v>45.97</v>
       </c>
+      <c r="F68" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1746,6 +1952,9 @@
       <c r="E69" t="n">
         <v>141.02</v>
       </c>
+      <c r="F69" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1754,15 +1963,18 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0</v>
+        <v>32.66</v>
       </c>
       <c r="C70" t="n">
         <v>23</v>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>7.51</v>
       </c>
       <c r="E70" t="n">
+        <v>40.17</v>
+      </c>
+      <c r="F70" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1773,15 +1985,18 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0</v>
+        <v>38.26</v>
       </c>
       <c r="C71" t="n">
         <v>23</v>
       </c>
       <c r="D71" t="n">
-        <v>0</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E71" t="n">
+        <v>47.06</v>
+      </c>
+      <c r="F71" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1792,16 +2007,19 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0</v>
+        <v>67.7</v>
       </c>
       <c r="C72" t="n">
         <v>23</v>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
+        <v>15.57</v>
       </c>
       <c r="E72" t="n">
-        <v>0</v>
+        <v>83.27</v>
+      </c>
+      <c r="F72" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -1811,15 +2029,18 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0</v>
+        <v>32.66</v>
       </c>
       <c r="C73" t="n">
         <v>23</v>
       </c>
       <c r="D73" t="n">
-        <v>0</v>
+        <v>7.51</v>
       </c>
       <c r="E73" t="n">
+        <v>40.17</v>
+      </c>
+      <c r="F73" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1830,15 +2051,18 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0</v>
+        <v>32.44</v>
       </c>
       <c r="C74" t="n">
         <v>23</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>7.46</v>
       </c>
       <c r="E74" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="F74" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1860,6 +2084,9 @@
       <c r="E75" t="n">
         <v>0</v>
       </c>
+      <c r="F75" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1868,15 +2095,18 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0</v>
+        <v>32.66</v>
       </c>
       <c r="C76" t="n">
         <v>23</v>
       </c>
       <c r="D76" t="n">
-        <v>0</v>
+        <v>7.51</v>
       </c>
       <c r="E76" t="n">
+        <v>40.17</v>
+      </c>
+      <c r="F76" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1898,6 +2128,9 @@
       <c r="E77" t="n">
         <v>0</v>
       </c>
+      <c r="F77" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1906,15 +2139,18 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0</v>
+        <v>27.5</v>
       </c>
       <c r="C78" t="n">
         <v>23</v>
       </c>
       <c r="D78" t="n">
-        <v>0</v>
+        <v>6.33</v>
       </c>
       <c r="E78" t="n">
+        <v>33.83</v>
+      </c>
+      <c r="F78" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1925,15 +2161,18 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0</v>
+        <v>32.75</v>
       </c>
       <c r="C79" t="n">
         <v>23</v>
       </c>
       <c r="D79" t="n">
-        <v>0</v>
+        <v>7.53</v>
       </c>
       <c r="E79" t="n">
+        <v>40.28</v>
+      </c>
+      <c r="F79" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1944,16 +2183,19 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0</v>
+        <v>89.2</v>
       </c>
       <c r="C80" t="n">
         <v>23</v>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
+        <v>20.52</v>
       </c>
       <c r="E80" t="n">
-        <v>0</v>
+        <v>109.72</v>
+      </c>
+      <c r="F80" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -1963,16 +2205,19 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0</v>
+        <v>89.2</v>
       </c>
       <c r="C81" t="n">
         <v>23</v>
       </c>
       <c r="D81" t="n">
-        <v>0</v>
+        <v>20.52</v>
       </c>
       <c r="E81" t="n">
-        <v>0</v>
+        <v>109.72</v>
+      </c>
+      <c r="F81" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -1993,6 +2238,9 @@
       <c r="E82" t="n">
         <v>0</v>
       </c>
+      <c r="F82" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2001,16 +2249,19 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0</v>
+        <v>1630</v>
       </c>
       <c r="C83" t="n">
         <v>23</v>
       </c>
       <c r="D83" t="n">
-        <v>0</v>
+        <v>374.9</v>
       </c>
       <c r="E83" t="n">
-        <v>0</v>
+        <v>2004.9</v>
+      </c>
+      <c r="F83" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -2031,6 +2282,9 @@
       <c r="E84" t="n">
         <v>0</v>
       </c>
+      <c r="F84" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2039,15 +2293,18 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0</v>
+        <v>32.75</v>
       </c>
       <c r="C85" t="n">
         <v>23</v>
       </c>
       <c r="D85" t="n">
-        <v>0</v>
+        <v>7.53</v>
       </c>
       <c r="E85" t="n">
+        <v>40.28</v>
+      </c>
+      <c r="F85" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2058,16 +2315,19 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0</v>
+        <v>206.83</v>
       </c>
       <c r="C86" t="n">
         <v>23</v>
       </c>
       <c r="D86" t="n">
-        <v>0</v>
+        <v>47.57</v>
       </c>
       <c r="E86" t="n">
-        <v>0</v>
+        <v>254.4</v>
+      </c>
+      <c r="F86" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -2077,15 +2337,18 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="C87" t="n">
         <v>23</v>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
+        <v>8.74</v>
       </c>
       <c r="E87" t="n">
+        <v>46.74</v>
+      </c>
+      <c r="F87" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2096,15 +2359,18 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0</v>
+        <v>32.75</v>
       </c>
       <c r="C88" t="n">
         <v>23</v>
       </c>
       <c r="D88" t="n">
-        <v>0</v>
+        <v>7.53</v>
       </c>
       <c r="E88" t="n">
+        <v>40.28</v>
+      </c>
+      <c r="F88" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2115,16 +2381,19 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0</v>
+        <v>89.2</v>
       </c>
       <c r="C89" t="n">
         <v>23</v>
       </c>
       <c r="D89" t="n">
-        <v>0</v>
+        <v>20.52</v>
       </c>
       <c r="E89" t="n">
-        <v>0</v>
+        <v>109.72</v>
+      </c>
+      <c r="F89" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -2134,15 +2403,18 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="C90" t="n">
         <v>23</v>
       </c>
       <c r="D90" t="n">
-        <v>0</v>
+        <v>8.74</v>
       </c>
       <c r="E90" t="n">
+        <v>46.74</v>
+      </c>
+      <c r="F90" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2153,15 +2425,18 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0</v>
+        <v>42.65</v>
       </c>
       <c r="C91" t="n">
         <v>23</v>
       </c>
       <c r="D91" t="n">
-        <v>0</v>
+        <v>9.81</v>
       </c>
       <c r="E91" t="n">
+        <v>52.46</v>
+      </c>
+      <c r="F91" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2172,16 +2447,19 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0</v>
+        <v>494.99</v>
       </c>
       <c r="C92" t="n">
         <v>23</v>
       </c>
       <c r="D92" t="n">
-        <v>0</v>
+        <v>113.85</v>
       </c>
       <c r="E92" t="n">
-        <v>0</v>
+        <v>608.84</v>
+      </c>
+      <c r="F92" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -2202,6 +2480,9 @@
       <c r="E93" t="n">
         <v>0</v>
       </c>
+      <c r="F93" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2219,6 +2500,9 @@
         <v>0</v>
       </c>
       <c r="E94" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📄 Update catalogo.xlsx from the app
</commit_message>
<xml_diff>
--- a/static/catalogo.xlsx
+++ b/static/catalogo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2506,6 +2506,28 @@
         <v>0</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>[Teste Pedro] Novo Produto</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" t="n">
+        <v>23</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>